<commit_message>
Update Register_Description sheet: HW write is higher priority for rwi
Matches the generator change in c93d89f. The sheet in CSR_Example.xlsx and
CSR_FORMAT_PROPOSAL.xlsx still said "Software write is higher priority".

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CSR_FORMAT_PROPOSAL.xlsx
+++ b/CSR_FORMAT_PROPOSAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27712"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\002_GitHub\APB-CSR-Generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\AppData\Roaming\MobaXterm\slash\RemoteFiles\264778_2_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE83735-1884-4388-9622-8E94304C9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A98CBD2-1CF6-4DEF-9A4D-82C9D45C9228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DE80DA28-ED5E-4F9B-81E9-F3E91ABAB1A9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DE80DA28-ED5E-4F9B-81E9-F3E91ABAB1A9}"/>
   </bookViews>
   <sheets>
     <sheet name="ASYNC_CSR" sheetId="6" r:id="rId1"/>
@@ -201,15 +201,9 @@
     <t>Read Write and Internal write</t>
   </si>
   <si>
-    <t>Software can write and read this register via APB, but this register also can be written by internal hardware signal. Software write is higher priority</t>
-  </si>
-  <si>
     <t>Write 1 to Clear</t>
   </si>
   <si>
-    <t>This register can be write by internal hardware signal and Software can write 1 to clear it value (clear to 0)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Register Type Introduction </t>
   </si>
   <si>
@@ -226,6 +220,12 @@
   </si>
   <si>
     <t>m_vlsi_async_csr</t>
+  </si>
+  <si>
+    <t>Software can write and read this register via APB, but this register also can be written by internal hardware signal. Hardware write is higher priority</t>
+  </si>
+  <si>
+    <t>This register can be write by internal hardware signal and Software can write 1 to clear it value (clear to 0). Hardware write is higher priority</t>
   </si>
 </sst>
 </file>
@@ -378,23 +378,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2487482</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>82252</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>224117</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>71718</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>605566</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>104552</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>478266</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>11654</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{266ADF93-ADC6-455D-2989-2CB6101AED0E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4ACDC73D-4DEB-37A9-978C-FE346EE1807A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -417,8 +417,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5499623" y="835287"/>
-          <a:ext cx="3487943" cy="7947100"/>
+          <a:off x="6284258" y="430306"/>
+          <a:ext cx="5059232" cy="9819042"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -758,23 +758,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1BE8D60-EEB2-4162-9272-A435C8FC0492}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -785,18 +785,18 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -807,7 +807,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -818,7 +818,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -829,7 +829,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -840,7 +840,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -851,13 +851,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
@@ -880,7 +880,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -895,7 +895,7 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
@@ -912,7 +912,7 @@
       </c>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
@@ -929,7 +929,7 @@
       </c>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
@@ -946,7 +946,7 @@
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
@@ -963,7 +963,7 @@
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
@@ -980,7 +980,7 @@
       </c>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
@@ -997,7 +997,7 @@
       </c>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
@@ -1122,23 +1122,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C536435B-4952-47A6-8C0D-14959CBB6C5F}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -1215,13 +1215,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
@@ -1486,43 +1486,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E03728AD-7351-4FF4-BFD8-5CD934512011}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="8"/>
-    <col min="2" max="2" width="26.81640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" style="8"/>
+    <col min="1" max="1" width="8.77734375" style="8"/>
+    <col min="2" max="2" width="26.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="8"/>
     <col min="4" max="4" width="44" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="8"/>
+    <col min="5" max="16384" width="8.77734375" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="7"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B2" s="7"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
-        <v>60</v>
-      </c>
       <c r="B3" s="7"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B5" s="9"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>46</v>
@@ -1534,7 +1534,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>1</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>2</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>3</v>
       </c>
@@ -1573,22 +1573,25 @@
         <v>26</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>4</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>44</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>55</v>
-      </c>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>